<commit_message>
pay for workers and add pays
</commit_message>
<xml_diff>
--- a/public/plantilla_trabajadores.xlsx
+++ b/public/plantilla_trabajadores.xlsx
@@ -407,10 +407,10 @@
         <v>Documento</v>
       </c>
       <c r="C1" t="str">
-        <v>Teléfono</v>
+        <v>Cargo</v>
       </c>
       <c r="D1" t="str">
-        <v>Cargo</v>
+        <v>Horas Trabajadas</v>
       </c>
       <c r="E1" t="str">
         <v>Horas Extras</v>
@@ -427,10 +427,10 @@
         <v>123456</v>
       </c>
       <c r="C2" t="str">
-        <v>300000000</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Operario</v>
+        <v>Cajero</v>
+      </c>
+      <c r="D2">
+        <v>80</v>
       </c>
       <c r="E2">
         <v>0</v>

</xml_diff>